<commit_message>
feat(server): support MCP UTF-8 text and structured Office editing
</commit_message>
<xml_diff>
--- a/apps/server/internal/office/templates/en-US/new.xlsx
+++ b/apps/server/internal/office/templates/en-US/new.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
+  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <x:workbookPr defaultThemeVersion="153222"/>
+  <x:bookViews>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </x:sheets>
+  <x:calcPr calcId="152511"/>
+  <x:extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+    </x:ext>
+  </x:extLst>
+</x:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -331,12 +331,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <x:dimension xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1"/>
+  <x:sheetFormatPr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:sheetData xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+  <x:printOptions xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headings="0" gridLines="0"/>
+  <x:pageMargins xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" paperSize="1" orientation="portrait" r:id="rId1"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(server): support MCP UTF-8 text and structured Office editing (#86)
* feat(server): support MCP UTF-8 text and structured Office editing

* fix(ci): copy officecli to system path and surface processing errors

* fix(mcp): refine text binary signatures and bind officecli flags
</commit_message>
<xml_diff>
--- a/apps/server/internal/office/templates/en-US/new.xlsx
+++ b/apps/server/internal/office/templates/en-US/new.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
+  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <x:workbookPr defaultThemeVersion="153222"/>
+  <x:bookViews>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </x:sheets>
+  <x:calcPr calcId="152511"/>
+  <x:extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+    </x:ext>
+  </x:extLst>
+</x:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -331,12 +331,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <x:dimension xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1"/>
+  <x:sheetFormatPr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:sheetData xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+  <x:printOptions xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headings="0" gridLines="0"/>
+  <x:pageMargins xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" paperSize="1" orientation="portrait" r:id="rId1"/>
+</x:worksheet>
 </file>
</xml_diff>